<commit_message>
Enhance quotes, discounts, and schedule availability
</commit_message>
<xml_diff>
--- a/docs/Disponibilidade_Cleaners_KACS.xlsx
+++ b/docs/Disponibilidade_Cleaners_KACS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor\OneDrive\Desktop\Trabalho\CODEX\Automacao\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA170BD-96AF-4D39-98BE-8B8769B417FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6355F6-DC67-49EE-9DB1-788C2E62082D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -765,11 +765,11 @@
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>12</v>
+      <c r="D13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>12</v>

</xml_diff>